<commit_message>
atualização no projeto de redes
</commit_message>
<xml_diff>
--- a/Redes/Documentação de Novas Máquinas.xlsx
+++ b/Redes/Documentação de Novas Máquinas.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="110">
   <si>
     <t>Equipamento</t>
   </si>
@@ -28,10 +28,19 @@
     <t>Máscara</t>
   </si>
   <si>
+    <t>VLANs</t>
+  </si>
+  <si>
     <t>Diretoria 1</t>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">Switch1= </t>
     </r>
     <r>
@@ -51,10 +60,19 @@
     <t>255.255.255.0</t>
   </si>
   <si>
+    <t>VLAN2</t>
+  </si>
+  <si>
     <t>Diretoria 2</t>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>Switch1=</t>
     </r>
     <r>
@@ -84,6 +102,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">Switch2= </t>
     </r>
     <r>
@@ -100,10 +124,19 @@
     <t>222.222.221.2</t>
   </si>
   <si>
+    <t>VLAN3</t>
+  </si>
+  <si>
     <t>Vendas 2</t>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">Switch2= </t>
     </r>
     <r>
@@ -124,6 +157,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">Switch2= </t>
     </r>
     <r>
@@ -144,6 +183,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">Switch2= </t>
     </r>
     <r>
@@ -160,10 +205,19 @@
     <t>222.222.224.2</t>
   </si>
   <si>
+    <t>VLAN4</t>
+  </si>
+  <si>
     <t>SAC 2</t>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">Switch2= </t>
     </r>
     <r>
@@ -184,6 +238,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">Switch3= </t>
     </r>
     <r>
@@ -200,10 +260,19 @@
     <t>222.222.223.2</t>
   </si>
   <si>
+    <t>VLAN5</t>
+  </si>
+  <si>
     <t>Servidor 2</t>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>Switch3=</t>
     </r>
     <r>
@@ -233,6 +302,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>Switch3=</t>
     </r>
     <r>
@@ -258,10 +333,19 @@
     <t>222.222.223.4</t>
   </si>
   <si>
+    <t>VLAN6</t>
+  </si>
+  <si>
     <t>Inovacao 1</t>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">Switch4= </t>
     </r>
     <r>
@@ -278,10 +362,19 @@
     <t>222.222.225.2</t>
   </si>
   <si>
+    <t>VLAN7</t>
+  </si>
+  <si>
     <t>Inovacao 2</t>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">Switch4= </t>
     </r>
     <r>
@@ -302,6 +395,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">Switch4= </t>
     </r>
     <r>
@@ -322,6 +421,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">Switch4= </t>
     </r>
     <r>
@@ -342,6 +447,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">Switch5= </t>
     </r>
     <r>
@@ -358,10 +469,19 @@
     <t>222.222.226.2</t>
   </si>
   <si>
+    <t>VLAN8</t>
+  </si>
+  <si>
     <t>Projeto 2</t>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">Switch5= </t>
     </r>
     <r>
@@ -382,6 +502,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">Switch5= </t>
     </r>
     <r>
@@ -402,6 +528,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">Switch5= </t>
     </r>
     <r>
@@ -418,10 +550,19 @@
     <t>222.222.227.2</t>
   </si>
   <si>
+    <t>VLAN9</t>
+  </si>
+  <si>
     <t>Design 2</t>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">Switch5= </t>
     </r>
     <r>
@@ -442,6 +583,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">Switch5= </t>
     </r>
     <r>
@@ -462,6 +609,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>Roteador=</t>
     </r>
     <r>
@@ -497,6 +650,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>Roteador=</t>
     </r>
     <r>
@@ -532,6 +691,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>Roteador=</t>
     </r>
     <r>
@@ -567,6 +732,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>Roteador=</t>
     </r>
     <r>
@@ -605,6 +776,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>Switch1</t>
     </r>
     <r>
@@ -664,6 +841,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">      </t>
     </r>
     <r>
@@ -723,6 +906,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>Switch1</t>
     </r>
     <r>
@@ -764,6 +953,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>Switch1</t>
     </r>
     <r>
@@ -808,6 +1003,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>Switch2</t>
     </r>
     <r>
@@ -867,6 +1068,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>Switch2</t>
     </r>
     <r>
@@ -917,6 +1124,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>Switch2</t>
     </r>
     <r>
@@ -967,6 +1180,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>Switch2</t>
     </r>
     <r>
@@ -1017,6 +1236,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>Switch2</t>
     </r>
     <r>
@@ -1070,6 +1295,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>Switch3</t>
     </r>
     <r>
@@ -1129,6 +1360,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>Switch3</t>
     </r>
     <r>
@@ -1188,6 +1425,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>Switch3</t>
     </r>
     <r>
@@ -1238,6 +1481,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>Switch3</t>
     </r>
     <r>
@@ -1291,6 +1540,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>Switch4</t>
     </r>
     <r>
@@ -1350,6 +1605,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>Switch4</t>
     </r>
     <r>
@@ -1409,6 +1670,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>Switch4</t>
     </r>
     <r>
@@ -1459,6 +1726,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>Switch4</t>
     </r>
     <r>
@@ -1512,6 +1785,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>Switch5</t>
     </r>
     <r>
@@ -1571,6 +1850,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>Switch5</t>
     </r>
     <r>
@@ -1621,6 +1906,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>Switch5</t>
     </r>
     <r>
@@ -1671,6 +1962,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>Switch5</t>
     </r>
     <r>
@@ -1721,6 +2018,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>Switch5</t>
     </r>
     <r>
@@ -1775,8 +2078,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="176" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="177" formatCode="_-&quot;R$&quot;\ * #,##0_-;\-&quot;R$&quot;\ * #,##0_-;_-&quot;R$&quot;\ * &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="176" formatCode="_-&quot;R$&quot;\ * #,##0_-;\-&quot;R$&quot;\ * #,##0_-;_-&quot;R$&quot;\ * &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="177" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="178" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="179" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
@@ -1809,36 +2112,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
@@ -1853,8 +2126,31 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1868,14 +2164,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <i/>
       <sz val="11"/>
       <color rgb="FF7F7F7F"/>
@@ -1884,8 +2172,32 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1906,6 +2218,13 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
@@ -1922,11 +2241,10 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color theme="3"/>
+      <color rgb="FF006100"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1936,21 +2254,6 @@
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="45">
     <fill>
@@ -2033,139 +2336,181 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="5" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="4" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2175,55 +2520,61 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -2244,15 +2595,6 @@
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
       <top style="thin">
         <color theme="4"/>
       </top>
@@ -2262,16 +2604,16 @@
       <diagonal/>
     </border>
     <border>
-      <left style="double">
+      <left style="thin">
         <color rgb="FF3F3F3F"/>
       </left>
-      <right style="double">
+      <right style="thin">
         <color rgb="FF3F3F3F"/>
       </right>
-      <top style="double">
+      <top style="thin">
         <color rgb="FF3F3F3F"/>
       </top>
-      <bottom style="double">
+      <bottom style="thin">
         <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
@@ -2300,181 +2642,157 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="20" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="32" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="30" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="29" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="31" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2493,14 +2811,17 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -2514,6 +2835,9 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -2523,6 +2847,9 @@
     <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -2532,8 +2859,8 @@
     <xf numFmtId="0" fontId="3" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2550,32 +2877,17 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -2896,16 +3208,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="B2:E48"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="12.75" outlineLevelCol="4"/>
+  <dimension ref="B2:F48"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="12.75" outlineLevelCol="5"/>
   <cols>
     <col min="2" max="2" width="12.7142857142857" customWidth="1"/>
     <col min="3" max="3" width="28.7142857142857" customWidth="1"/>
     <col min="4" max="4" width="15.5714285714286" customWidth="1"/>
     <col min="5" max="5" width="19.8571428571429" customWidth="1"/>
+    <col min="7" max="7" width="23.2857142857143" customWidth="1"/>
+    <col min="9" max="9" width="8.71428571428571" customWidth="1"/>
+    <col min="10" max="10" width="7.28571428571429" customWidth="1"/>
+    <col min="11" max="11" width="6.42857142857143" customWidth="1"/>
+    <col min="12" max="12" width="11.5714285714286" customWidth="1"/>
+    <col min="13" max="13" width="8.85714285714286" customWidth="1"/>
+    <col min="14" max="14" width="7.28571428571429" customWidth="1"/>
+    <col min="15" max="15" width="6.85714285714286" customWidth="1"/>
+    <col min="16" max="16" width="7.42857142857143" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:5">
+    <row r="2" spans="2:6">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -2918,525 +3239,564 @@
       <c r="E2" s="2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" ht="13.5" spans="2:5">
+      <c r="F2" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" ht="13.5" spans="2:6">
       <c r="B3" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" ht="13.5" spans="2:5">
+        <v>8</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" ht="13.5" spans="2:6">
       <c r="B4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" ht="13.5" spans="2:5">
-      <c r="B5" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" s="7" t="s">
+      <c r="F4" s="6"/>
+    </row>
+    <row r="5" ht="13.5" spans="2:6">
+      <c r="B5" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="7" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" ht="13.5" spans="2:5">
-      <c r="B6" s="6" t="s">
+      <c r="C5" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="D5" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="E5" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="E6" s="7" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" ht="13.5" spans="2:5">
-      <c r="B7" s="6" t="s">
+    </row>
+    <row r="6" ht="13.5" spans="2:6">
+      <c r="B6" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C6" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D6" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="7" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" ht="13.5" spans="2:5">
-      <c r="B8" s="6" t="s">
+      <c r="E6" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="9"/>
+    </row>
+    <row r="7" ht="13.5" spans="2:6">
+      <c r="B7" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C7" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D7" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="E8" s="7" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" ht="13.5" spans="2:5">
-      <c r="B9" s="6" t="s">
+      <c r="E7" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="9"/>
+    </row>
+    <row r="8" ht="13.5" spans="2:6">
+      <c r="B8" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C8" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D8" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="E9" s="7" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" ht="13.5" spans="2:5">
-      <c r="B10" s="10" t="s">
+      <c r="E8" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="10" t="s">
+    </row>
+    <row r="9" ht="13.5" spans="2:6">
+      <c r="B9" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="C9" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="E10" s="12" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" ht="13.5" spans="2:5">
-      <c r="B11" s="10" t="s">
+      <c r="D9" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="E9" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9" s="9"/>
+    </row>
+    <row r="10" ht="13.5" spans="2:6">
+      <c r="B10" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="C10" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="E11" s="12" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="12" ht="13.5" spans="2:5">
-      <c r="B12" s="10" t="s">
+      <c r="D10" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="E10" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="F10" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="D12" s="11" t="s">
+    </row>
+    <row r="11" ht="13.5" spans="2:6">
+      <c r="B11" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="E12" s="12" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="13" ht="13.5" spans="2:5">
-      <c r="B13" s="13" t="s">
+      <c r="C11" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="C13" s="13" t="s">
+      <c r="D11" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="D13" s="14" t="s">
+      <c r="E11" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="F11" s="14"/>
+    </row>
+    <row r="12" ht="13.5" spans="2:6">
+      <c r="B12" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="E13" s="15" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="14" ht="13.5" spans="2:5">
-      <c r="B14" s="13" t="s">
+      <c r="C12" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="C14" s="13" t="s">
+      <c r="D12" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="D14" s="14" t="s">
+      <c r="E12" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="E14" s="15" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="15" ht="13.5" spans="2:5">
-      <c r="B15" s="13" t="s">
+    </row>
+    <row r="13" ht="13.5" spans="2:6">
+      <c r="B13" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="C15" s="13" t="s">
+      <c r="C13" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="D15" s="14" t="s">
+      <c r="D13" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="E15" s="15" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="16" ht="13.5" spans="2:5">
-      <c r="B16" s="13" t="s">
+      <c r="E13" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="F13" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="C16" s="13" t="s">
+    </row>
+    <row r="14" ht="13.5" spans="2:6">
+      <c r="B14" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="D16" s="14" t="s">
+      <c r="C14" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E16" s="15" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="17" ht="13.5" spans="2:5">
-      <c r="B17" s="16" t="s">
+      <c r="D14" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="C17" s="16" t="s">
+      <c r="E14" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="F14" s="18"/>
+    </row>
+    <row r="15" ht="13.5" spans="2:6">
+      <c r="B15" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="D17" s="17" t="s">
+      <c r="C15" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="E17" s="18" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="18" ht="13.5" spans="2:5">
-      <c r="B18" s="16" t="s">
+      <c r="D15" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="C18" s="16" t="s">
+      <c r="E15" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="F15" s="18"/>
+    </row>
+    <row r="16" ht="13.5" spans="2:6">
+      <c r="B16" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="D18" s="17" t="s">
+      <c r="C16" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="E18" s="18" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="19" ht="13.5" spans="2:5">
-      <c r="B19" s="16" t="s">
+      <c r="D16" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="C19" s="16" t="s">
+      <c r="E16" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" s="18"/>
+    </row>
+    <row r="17" ht="13.5" spans="2:6">
+      <c r="B17" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="D19" s="17" t="s">
+      <c r="C17" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="E19" s="18" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="20" ht="13.5" spans="2:5">
-      <c r="B20" s="16" t="s">
+      <c r="D17" s="20" t="s">
         <v>56</v>
       </c>
+      <c r="E17" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="F17" s="22" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="18" ht="13.5" spans="2:6">
+      <c r="B18" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="C18" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="D18" s="20" t="s">
+        <v>60</v>
+      </c>
+      <c r="E18" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="F18" s="22"/>
+    </row>
+    <row r="19" ht="13.5" spans="2:6">
+      <c r="B19" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="C19" s="19" t="s">
+        <v>62</v>
+      </c>
+      <c r="D19" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="E19" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="F19" s="22"/>
+    </row>
+    <row r="20" ht="13.5" spans="2:6">
+      <c r="B20" s="19" t="s">
+        <v>64</v>
+      </c>
       <c r="C20" s="19" t="s">
-        <v>57</v>
-      </c>
-      <c r="D20" s="17" t="s">
-        <v>58</v>
-      </c>
-      <c r="E20" s="18" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="21" ht="13.5" spans="2:5">
-      <c r="B21" s="16" t="s">
-        <v>59</v>
+        <v>65</v>
+      </c>
+      <c r="D20" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="E20" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" s="22" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="21" ht="13.5" spans="2:6">
+      <c r="B21" s="19" t="s">
+        <v>68</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>60</v>
-      </c>
-      <c r="D21" s="17" t="s">
-        <v>61</v>
-      </c>
-      <c r="E21" s="18" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="22" ht="13.5" spans="2:5">
-      <c r="B22" s="16" t="s">
-        <v>62</v>
+        <v>69</v>
+      </c>
+      <c r="D21" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="E21" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="F21" s="22"/>
+    </row>
+    <row r="22" ht="13.5" spans="2:6">
+      <c r="B22" s="19" t="s">
+        <v>71</v>
       </c>
       <c r="C22" s="19" t="s">
-        <v>63</v>
-      </c>
-      <c r="D22" s="17" t="s">
-        <v>64</v>
-      </c>
-      <c r="E22" s="18" t="s">
-        <v>7</v>
-      </c>
+        <v>72</v>
+      </c>
+      <c r="D22" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="E22" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="F22" s="22"/>
     </row>
     <row r="23" ht="27" spans="2:5">
-      <c r="B23" s="20" t="s">
-        <v>65</v>
-      </c>
-      <c r="C23" s="21" t="s">
-        <v>66</v>
-      </c>
-      <c r="D23" s="22" t="s">
-        <v>67</v>
-      </c>
-      <c r="E23" s="23">
+      <c r="B23" s="23" t="s">
+        <v>74</v>
+      </c>
+      <c r="C23" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="D23" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="E23" s="26">
         <v>255255255252</v>
       </c>
     </row>
     <row r="24" ht="27" spans="2:5">
-      <c r="B24" s="20"/>
-      <c r="C24" s="21" t="s">
-        <v>68</v>
-      </c>
-      <c r="D24" s="22" t="s">
-        <v>69</v>
-      </c>
-      <c r="E24" s="22" t="s">
-        <v>7</v>
+      <c r="B24" s="23"/>
+      <c r="C24" s="24" t="s">
+        <v>77</v>
+      </c>
+      <c r="D24" s="25" t="s">
+        <v>78</v>
+      </c>
+      <c r="E24" s="25" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="25" ht="27" spans="2:5">
-      <c r="B25" s="20"/>
-      <c r="C25" s="21" t="s">
-        <v>70</v>
-      </c>
-      <c r="D25" s="22" t="s">
-        <v>71</v>
-      </c>
-      <c r="E25" s="22" t="s">
-        <v>7</v>
+      <c r="B25" s="23"/>
+      <c r="C25" s="24" t="s">
+        <v>79</v>
+      </c>
+      <c r="D25" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="E25" s="25" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="26" ht="27" spans="2:5">
-      <c r="B26" s="20"/>
-      <c r="C26" s="21" t="s">
-        <v>72</v>
-      </c>
-      <c r="D26" s="22" t="s">
-        <v>73</v>
-      </c>
-      <c r="E26" s="22" t="s">
-        <v>7</v>
+      <c r="B26" s="23"/>
+      <c r="C26" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="D26" s="25" t="s">
+        <v>82</v>
+      </c>
+      <c r="E26" s="25" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="27" spans="2:5">
-      <c r="B27" s="24" t="s">
-        <v>74</v>
-      </c>
-      <c r="C27" s="25" t="s">
-        <v>75</v>
-      </c>
-      <c r="D27" s="25"/>
-      <c r="E27" s="25"/>
+      <c r="B27" s="27" t="s">
+        <v>83</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
     </row>
     <row r="28" spans="2:5">
-      <c r="B28" s="24"/>
-      <c r="C28" s="25" t="s">
-        <v>76</v>
-      </c>
-      <c r="D28" s="25"/>
-      <c r="E28" s="25"/>
+      <c r="B28" s="27"/>
+      <c r="C28" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
     </row>
     <row r="29" spans="2:5">
-      <c r="B29" s="24"/>
-      <c r="C29" s="25" t="s">
-        <v>77</v>
-      </c>
-      <c r="D29" s="25"/>
-      <c r="E29" s="25"/>
+      <c r="B29" s="27"/>
+      <c r="C29" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
     </row>
     <row r="30" spans="2:5">
-      <c r="B30" s="24"/>
-      <c r="C30" s="25" t="s">
-        <v>78</v>
-      </c>
-      <c r="D30" s="25"/>
-      <c r="E30" s="25"/>
+      <c r="B30" s="27"/>
+      <c r="C30" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="D30" s="3"/>
+      <c r="E30" s="3"/>
     </row>
     <row r="31" spans="2:5">
-      <c r="B31" s="26" t="s">
-        <v>79</v>
-      </c>
-      <c r="C31" s="27" t="s">
-        <v>80</v>
-      </c>
-      <c r="D31" s="27"/>
-      <c r="E31" s="27"/>
+      <c r="B31" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="C31" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="D31" s="7"/>
+      <c r="E31" s="7"/>
     </row>
     <row r="32" spans="2:5">
-      <c r="B32" s="26"/>
-      <c r="C32" s="27" t="s">
-        <v>81</v>
-      </c>
-      <c r="D32" s="27"/>
-      <c r="E32" s="27"/>
+      <c r="B32" s="28"/>
+      <c r="C32" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="D32" s="7"/>
+      <c r="E32" s="7"/>
     </row>
     <row r="33" spans="2:5">
-      <c r="B33" s="26"/>
-      <c r="C33" s="27" t="s">
-        <v>82</v>
-      </c>
-      <c r="D33" s="27"/>
-      <c r="E33" s="27"/>
+      <c r="B33" s="28"/>
+      <c r="C33" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="D33" s="7"/>
+      <c r="E33" s="7"/>
     </row>
     <row r="34" spans="2:5">
-      <c r="B34" s="26"/>
-      <c r="C34" s="27" t="s">
-        <v>83</v>
-      </c>
-      <c r="D34" s="27"/>
-      <c r="E34" s="27"/>
+      <c r="B34" s="28"/>
+      <c r="C34" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="D34" s="7"/>
+      <c r="E34" s="7"/>
     </row>
     <row r="35" spans="2:5">
-      <c r="B35" s="26"/>
-      <c r="C35" s="27" t="s">
-        <v>84</v>
-      </c>
-      <c r="D35" s="27"/>
-      <c r="E35" s="27"/>
+      <c r="B35" s="28"/>
+      <c r="C35" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="D35" s="7"/>
+      <c r="E35" s="7"/>
     </row>
     <row r="36" spans="2:5">
-      <c r="B36" s="28" t="s">
-        <v>85</v>
-      </c>
-      <c r="C36" s="29" t="s">
-        <v>86</v>
-      </c>
-      <c r="D36" s="29"/>
-      <c r="E36" s="29"/>
+      <c r="B36" s="29" t="s">
+        <v>94</v>
+      </c>
+      <c r="C36" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="D36" s="11"/>
+      <c r="E36" s="11"/>
     </row>
     <row r="37" spans="2:5">
-      <c r="B37" s="28"/>
-      <c r="C37" s="29" t="s">
-        <v>87</v>
-      </c>
-      <c r="D37" s="29"/>
-      <c r="E37" s="29"/>
+      <c r="B37" s="29"/>
+      <c r="C37" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="D37" s="11"/>
+      <c r="E37" s="11"/>
     </row>
     <row r="38" spans="2:5">
-      <c r="B38" s="28"/>
-      <c r="C38" s="29" t="s">
-        <v>88</v>
-      </c>
-      <c r="D38" s="29"/>
-      <c r="E38" s="29"/>
+      <c r="B38" s="29"/>
+      <c r="C38" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="D38" s="11"/>
+      <c r="E38" s="11"/>
     </row>
     <row r="39" spans="2:5">
-      <c r="B39" s="28"/>
-      <c r="C39" s="29" t="s">
-        <v>89</v>
-      </c>
-      <c r="D39" s="29"/>
-      <c r="E39" s="29"/>
+      <c r="B39" s="29"/>
+      <c r="C39" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="D39" s="11"/>
+      <c r="E39" s="11"/>
     </row>
     <row r="40" spans="2:5">
       <c r="B40" s="30" t="s">
-        <v>90</v>
-      </c>
-      <c r="C40" s="31" t="s">
-        <v>91</v>
-      </c>
-      <c r="D40" s="31"/>
-      <c r="E40" s="31"/>
+        <v>99</v>
+      </c>
+      <c r="C40" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="D40" s="15"/>
+      <c r="E40" s="15"/>
     </row>
     <row r="41" spans="2:5">
       <c r="B41" s="30"/>
-      <c r="C41" s="31" t="s">
-        <v>92</v>
-      </c>
-      <c r="D41" s="31"/>
-      <c r="E41" s="31"/>
+      <c r="C41" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="D41" s="15"/>
+      <c r="E41" s="15"/>
     </row>
     <row r="42" spans="2:5">
       <c r="B42" s="30"/>
-      <c r="C42" s="31" t="s">
-        <v>93</v>
-      </c>
-      <c r="D42" s="31"/>
-      <c r="E42" s="31"/>
+      <c r="C42" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="D42" s="15"/>
+      <c r="E42" s="15"/>
     </row>
     <row r="43" spans="2:5">
       <c r="B43" s="30"/>
-      <c r="C43" s="31" t="s">
-        <v>94</v>
-      </c>
-      <c r="D43" s="31"/>
-      <c r="E43" s="31"/>
+      <c r="C43" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="D43" s="15"/>
+      <c r="E43" s="15"/>
     </row>
     <row r="44" spans="2:5">
-      <c r="B44" s="32" t="s">
-        <v>95</v>
-      </c>
-      <c r="C44" s="33" t="s">
-        <v>96</v>
-      </c>
-      <c r="D44" s="33"/>
-      <c r="E44" s="33"/>
+      <c r="B44" s="31" t="s">
+        <v>104</v>
+      </c>
+      <c r="C44" s="19" t="s">
+        <v>105</v>
+      </c>
+      <c r="D44" s="19"/>
+      <c r="E44" s="19"/>
     </row>
     <row r="45" spans="2:5">
-      <c r="B45" s="32"/>
-      <c r="C45" s="33" t="s">
-        <v>97</v>
-      </c>
-      <c r="D45" s="33"/>
-      <c r="E45" s="33"/>
+      <c r="B45" s="31"/>
+      <c r="C45" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="D45" s="19"/>
+      <c r="E45" s="19"/>
     </row>
     <row r="46" spans="2:5">
-      <c r="B46" s="32"/>
-      <c r="C46" s="33" t="s">
-        <v>98</v>
-      </c>
-      <c r="D46" s="33"/>
-      <c r="E46" s="33"/>
+      <c r="B46" s="31"/>
+      <c r="C46" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="D46" s="19"/>
+      <c r="E46" s="19"/>
     </row>
     <row r="47" spans="2:5">
-      <c r="B47" s="32"/>
-      <c r="C47" s="33" t="s">
-        <v>99</v>
-      </c>
-      <c r="D47" s="33"/>
-      <c r="E47" s="33"/>
+      <c r="B47" s="31"/>
+      <c r="C47" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="D47" s="19"/>
+      <c r="E47" s="19"/>
     </row>
     <row r="48" spans="2:5">
-      <c r="B48" s="32"/>
-      <c r="C48" s="33" t="s">
-        <v>100</v>
-      </c>
-      <c r="D48" s="33"/>
-      <c r="E48" s="33"/>
+      <c r="B48" s="31"/>
+      <c r="C48" s="19" t="s">
+        <v>109</v>
+      </c>
+      <c r="D48" s="19"/>
+      <c r="E48" s="19"/>
     </row>
   </sheetData>
-  <mergeCells count="28">
+  <mergeCells count="35">
     <mergeCell ref="C27:E27"/>
     <mergeCell ref="C28:E28"/>
     <mergeCell ref="C29:E29"/>
@@ -3465,6 +3825,13 @@
     <mergeCell ref="B36:B39"/>
     <mergeCell ref="B40:B43"/>
     <mergeCell ref="B44:B48"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="F5:F7"/>
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="F10:F11"/>
+    <mergeCell ref="F13:F16"/>
+    <mergeCell ref="F17:F19"/>
+    <mergeCell ref="F20:F22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>